<commit_message>
Add Test case ChecKout
</commit_message>
<xml_diff>
--- a/saucedemo/Test cases.xlsx
+++ b/saucedemo/Test cases.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MOHAMED\job\Software Testing [ QA ]\Projects\saucedemo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99FC663A-E3E7-4E2A-BA26-FE5C96BF290B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E09CDB86-30AF-4ACF-A130-0082746E005C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" activeTab="2" xr2:uid="{A007FA3B-5C3E-4B15-A9AC-45DC79D3E82D}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" activeTab="3" xr2:uid="{A007FA3B-5C3E-4B15-A9AC-45DC79D3E82D}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
     <sheet name="Product page" sheetId="2" r:id="rId2"/>
     <sheet name="Cart" sheetId="3" r:id="rId3"/>
+    <sheet name="CheckOut" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="171">
   <si>
     <t>Test Scenario</t>
   </si>
@@ -571,6 +572,66 @@
   </si>
   <si>
     <t>The Filter does not working</t>
+  </si>
+  <si>
+    <t>CheckOut</t>
+  </si>
+  <si>
+    <t>CO001</t>
+  </si>
+  <si>
+    <t>CO002</t>
+  </si>
+  <si>
+    <t>CO003</t>
+  </si>
+  <si>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>Verify error msg when user enters Empty data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1- Open the product page
+2- Open the  Cart page
+3- Click the Contino button </t>
+  </si>
+  <si>
+    <t>Verify that the Last Name field accepts text input</t>
+  </si>
+  <si>
+    <t>LastName field</t>
+  </si>
+  <si>
+    <t>1-Login to the application.
+2-Add a product to the cart.
+3-Proceed to Checkout.
+4-Enter a valid First Name.
+5-Click the Last Name field.
+6-Enter a valid Last Name.</t>
+  </si>
+  <si>
+    <t>The Last Name field accepts text input</t>
+  </si>
+  <si>
+    <t>The Last Name field does not accept text input</t>
+  </si>
+  <si>
+    <t>Cancel</t>
+  </si>
+  <si>
+    <t>Verify that clicking Cancel returns the user to the Cart page</t>
+  </si>
+  <si>
+    <t>1-Open the Cart page.
+2-Click Checkout.
+3-Click the Cancel button.</t>
+  </si>
+  <si>
+    <t>The user is redirected to the Cart page</t>
+  </si>
+  <si>
+    <t>The user was redirected to the Cart page successfully</t>
   </si>
 </sst>
 </file>
@@ -1468,7 +1529,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FFEAE05-2AA3-4904-928B-B110F353CA3B}">
-  <dimension ref="H9:S26"/>
+  <dimension ref="I9:S26"/>
   <sheetFormatPr defaultColWidth="65.5546875" defaultRowHeight="99.6" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="9" max="9" width="31.5546875" customWidth="1"/>
@@ -1484,7 +1545,7 @@
     <col min="19" max="19" width="33.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="9" spans="8:19" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="9:19" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I9" s="8" t="s">
         <v>0</v>
       </c>
@@ -1519,7 +1580,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="8:19" ht="99.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="9:19" ht="99.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I10" s="19" t="s">
         <v>66</v>
       </c>
@@ -1554,7 +1615,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="8:19" ht="99.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="9:19" ht="99.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I11" s="20"/>
       <c r="J11" s="1" t="s">
         <v>125</v>
@@ -1587,7 +1648,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="8:19" ht="99.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="9:19" ht="99.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I12" s="20"/>
       <c r="J12" s="1" t="s">
         <v>126</v>
@@ -1620,7 +1681,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="8:19" ht="99.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="9:19" ht="99.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I13" s="20"/>
       <c r="J13" s="1" t="s">
         <v>127</v>
@@ -1653,7 +1714,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="8:19" ht="99.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="9:19" ht="99.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I14" s="21" t="s">
         <v>70</v>
       </c>
@@ -1686,7 +1747,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="8:19" ht="99.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="9:19" ht="99.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I15" s="21"/>
       <c r="J15" s="1" t="s">
         <v>129</v>
@@ -1717,11 +1778,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="8:19" ht="99.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H16">
-        <f ca="1">H10:H16</f>
-        <v>0</v>
-      </c>
+    <row r="16" spans="9:19" ht="99.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I16" s="21"/>
       <c r="J16" s="1" t="s">
         <v>130</v>
@@ -2225,4 +2282,160 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9643AE81-234F-4341-BDB5-25B9CA2D02D5}">
+  <dimension ref="D1:N7"/>
+  <sheetFormatPr defaultColWidth="23.44140625" defaultRowHeight="62.4" customHeight="1" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="4" max="4" width="21.21875" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" customWidth="1"/>
+    <col min="6" max="6" width="18.88671875" customWidth="1"/>
+    <col min="7" max="7" width="61.21875" customWidth="1"/>
+    <col min="8" max="8" width="46" customWidth="1"/>
+    <col min="9" max="9" width="28.21875" customWidth="1"/>
+    <col min="11" max="11" width="35.33203125" customWidth="1"/>
+    <col min="12" max="12" width="46.109375" customWidth="1"/>
+    <col min="13" max="13" width="20.44140625" customWidth="1"/>
+    <col min="14" max="14" width="19.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="4:14" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="4:14" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="4:14" ht="65.400000000000006" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="4:14" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D4" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="M4" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="N4" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="4:14" ht="84" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D5" s="23" t="s">
+        <v>154</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="I5" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="J5" s="13"/>
+      <c r="K5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="4:14" ht="96" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D6" s="23"/>
+      <c r="E6" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F6" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="I6" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="4:14" ht="62.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D7" s="23"/>
+      <c r="E7" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>166</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="L7" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="M7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="N7" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="D5:D7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>